<commit_message>
Added template reader, models.py
Added template reader to separate logic from template writer. Also added models.py to effectively store data in dataclasses rather than pure json - allowing for hierarchical structure.
</commit_message>
<xml_diff>
--- a/data/templates/Ram 2026_Owen Testing.xlsx
+++ b/data/templates/Ram 2026_Owen Testing.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -2292,6 +2292,12 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2300,21 +2306,6 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2333,6 +2324,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2962,10 +2962,10 @@
       <c r="U7" s="14"/>
     </row>
     <row r="8" spans="1:77" x14ac:dyDescent="0.25">
-      <c r="A8" s="144" t="s">
+      <c r="A8" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="145"/>
+      <c r="B8" s="139"/>
       <c r="C8" s="78"/>
       <c r="D8" s="83" t="s">
         <v>8</v>
@@ -3052,106 +3052,106 @@
       <c r="I13" s="68"/>
       <c r="J13" s="68"/>
       <c r="K13" s="72"/>
-      <c r="L13" s="146" t="s">
+      <c r="L13" s="143" t="s">
         <v>14</v>
       </c>
-      <c r="M13" s="147"/>
-      <c r="N13" s="138" cm="1">
+      <c r="M13" s="144"/>
+      <c r="N13" s="140" cm="1">
         <f t="array" ref="N13">SUM(Q17:Q65)+SUM(_xlfn._xlws.FILTER(P17:P65,Q17:Q65=""))+SUM(_xlfn._xlws.FILTER(O17:O65,(P17:P65="")*(Q17:Q65="")))+SUMIFS(R17:R65,Q17:Q65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(N17:N65)</f>
         <v>685594.25000000012</v>
       </c>
-      <c r="O13" s="139"/>
-      <c r="P13" s="139"/>
-      <c r="Q13" s="139"/>
-      <c r="R13" s="140"/>
-      <c r="S13" s="138" cm="1">
+      <c r="O13" s="141"/>
+      <c r="P13" s="141"/>
+      <c r="Q13" s="141"/>
+      <c r="R13" s="142"/>
+      <c r="S13" s="140" cm="1">
         <f t="array" ref="S13">SUM(V17:V65)+SUM(_xlfn._xlws.FILTER(U17:U65,V17:V65=""))+SUM(_xlfn._xlws.FILTER(T17:T65,(U17:U65="")*(V17:V65="")))+SUMIFS(W17:W65,V17:V65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(S17:S65)</f>
         <v>891985.88</v>
       </c>
-      <c r="T13" s="139"/>
-      <c r="U13" s="139"/>
-      <c r="V13" s="139"/>
-      <c r="W13" s="140"/>
-      <c r="X13" s="138" cm="1">
+      <c r="T13" s="141"/>
+      <c r="U13" s="141"/>
+      <c r="V13" s="141"/>
+      <c r="W13" s="142"/>
+      <c r="X13" s="140" cm="1">
         <f t="array" ref="X13">SUM(AA17:AA65)+SUM(_xlfn._xlws.FILTER(Z17:Z65,AA17:AA65=""))+SUM(_xlfn._xlws.FILTER(Y17:Y65,(Z17:Z65="")*(AA17:AA65="")))+SUMIFS(AB17:AB65,AA17:AA65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(X17:X65)</f>
         <v>647579.66999999993</v>
       </c>
-      <c r="Y13" s="139"/>
-      <c r="Z13" s="139"/>
-      <c r="AA13" s="139"/>
-      <c r="AB13" s="140"/>
-      <c r="AC13" s="138" cm="1">
+      <c r="Y13" s="141"/>
+      <c r="Z13" s="141"/>
+      <c r="AA13" s="141"/>
+      <c r="AB13" s="142"/>
+      <c r="AC13" s="140" cm="1">
         <f t="array" ref="AC13">SUM(AF17:AF65)+SUM(_xlfn._xlws.FILTER(AE17:AE65,AF17:AF65=""))+SUM(_xlfn._xlws.FILTER(AD17:AD65,(AE17:AE65="")*(AF17:AF65="")))+SUMIFS(AG17:AG65,AF17:AF65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AC17:AC65)</f>
         <v>647579.66999999993</v>
       </c>
-      <c r="AD13" s="139"/>
-      <c r="AE13" s="139"/>
-      <c r="AF13" s="139"/>
-      <c r="AG13" s="140"/>
-      <c r="AH13" s="138" cm="1">
+      <c r="AD13" s="141"/>
+      <c r="AE13" s="141"/>
+      <c r="AF13" s="141"/>
+      <c r="AG13" s="142"/>
+      <c r="AH13" s="140" cm="1">
         <f t="array" ref="AH13">SUM(AK17:AK65)+SUM(_xlfn._xlws.FILTER(AJ17:AJ65,AK17:AK65=""))+SUM(_xlfn._xlws.FILTER(AI17:AI65,(AJ17:AJ65="")*(AK17:AK65="")))+SUMIFS(AL17:AL65,AK17:AK65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AH17:AH65)</f>
         <v>645269.66999999993</v>
       </c>
-      <c r="AI13" s="139"/>
-      <c r="AJ13" s="139"/>
-      <c r="AK13" s="139"/>
-      <c r="AL13" s="140"/>
-      <c r="AM13" s="138" cm="1">
+      <c r="AI13" s="141"/>
+      <c r="AJ13" s="141"/>
+      <c r="AK13" s="141"/>
+      <c r="AL13" s="142"/>
+      <c r="AM13" s="140" cm="1">
         <f t="array" ref="AM13">SUM(AP17:AP65)+SUM(_xlfn._xlws.FILTER(AO17:AO65,AP17:AP65=""))+SUM(_xlfn._xlws.FILTER(AN17:AN65,(AO17:AO65="")*(AP17:AP65="")))+SUMIFS(AQ17:AQ65,AP17:AP65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AM17:AM65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AN13" s="139"/>
-      <c r="AO13" s="139"/>
-      <c r="AP13" s="139"/>
-      <c r="AQ13" s="140"/>
-      <c r="AR13" s="138" cm="1">
+      <c r="AN13" s="141"/>
+      <c r="AO13" s="141"/>
+      <c r="AP13" s="141"/>
+      <c r="AQ13" s="142"/>
+      <c r="AR13" s="140" cm="1">
         <f t="array" ref="AR13">SUM(AU17:AU65)+SUM(_xlfn._xlws.FILTER(AT17:AT65,AU17:AU65=""))+SUM(_xlfn._xlws.FILTER(AS17:AS65,(AT17:AT65="")*(AU17:AU65="")))+SUMIFS(AV17:AV65,AU17:AU65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AR17:AR65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AS13" s="139"/>
-      <c r="AT13" s="139"/>
-      <c r="AU13" s="139"/>
-      <c r="AV13" s="140"/>
-      <c r="AW13" s="138" cm="1">
+      <c r="AS13" s="141"/>
+      <c r="AT13" s="141"/>
+      <c r="AU13" s="141"/>
+      <c r="AV13" s="142"/>
+      <c r="AW13" s="140" cm="1">
         <f t="array" ref="AW13">SUM(AZ17:AZ65)+SUM(_xlfn._xlws.FILTER(AY17:AY65,AZ17:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX17:AX65,(AY17:AY65="")*(AZ17:AZ65="")))+SUMIFS(BA17:BA65,AZ17:AZ65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AW17:AW65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AX13" s="139"/>
-      <c r="AY13" s="139"/>
-      <c r="AZ13" s="139"/>
-      <c r="BA13" s="140"/>
-      <c r="BB13" s="138" cm="1">
+      <c r="AX13" s="141"/>
+      <c r="AY13" s="141"/>
+      <c r="AZ13" s="141"/>
+      <c r="BA13" s="142"/>
+      <c r="BB13" s="140" cm="1">
         <f t="array" ref="BB13">SUM(BE17:BE65)+SUM(_xlfn._xlws.FILTER(BD17:BD65,BE17:BE65=""))+SUM(_xlfn._xlws.FILTER(BC17:BC65,(BD17:BD65="")*(BE17:BE65="")))+SUMIFS(BF17:BF65,BE17:BE65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BB17:BB65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BC13" s="139"/>
-      <c r="BD13" s="139"/>
-      <c r="BE13" s="139"/>
-      <c r="BF13" s="140"/>
-      <c r="BG13" s="138" cm="1">
+      <c r="BC13" s="141"/>
+      <c r="BD13" s="141"/>
+      <c r="BE13" s="141"/>
+      <c r="BF13" s="142"/>
+      <c r="BG13" s="140" cm="1">
         <f t="array" ref="BG13">SUM(BJ17:BJ65)+SUM(_xlfn._xlws.FILTER(BI17:BI65,BJ17:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH17:BH65,(BI17:BI65="")*(BJ17:BJ65="")))+SUMIFS(BK17:BK65,BJ17:BJ65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BG17:BG65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BH13" s="139"/>
-      <c r="BI13" s="139"/>
-      <c r="BJ13" s="139"/>
-      <c r="BK13" s="140"/>
-      <c r="BL13" s="138" cm="1">
+      <c r="BH13" s="141"/>
+      <c r="BI13" s="141"/>
+      <c r="BJ13" s="141"/>
+      <c r="BK13" s="142"/>
+      <c r="BL13" s="140" cm="1">
         <f t="array" ref="BL13">SUM(BO17:BO65)+SUM(_xlfn._xlws.FILTER(BN17:BN65,BO17:BO65=""))+SUM(_xlfn._xlws.FILTER(BM17:BM65,(BN17:BN65="")*(BO17:BO65="")))+SUMIFS(BP17:BP65,BO17:BO65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BL17:BL65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BM13" s="139"/>
-      <c r="BN13" s="139"/>
-      <c r="BO13" s="139"/>
-      <c r="BP13" s="140"/>
-      <c r="BQ13" s="138" cm="1">
+      <c r="BM13" s="141"/>
+      <c r="BN13" s="141"/>
+      <c r="BO13" s="141"/>
+      <c r="BP13" s="142"/>
+      <c r="BQ13" s="140" cm="1">
         <f t="array" ref="BQ13">SUM(BT17:BT65)+SUM(_xlfn._xlws.FILTER(BS17:BS65,BT17:BT65=""))+SUM(_xlfn._xlws.FILTER(BR17:BR65,(BS17:BS65="")*(BT17:BT65="")))+SUMIFS(BU17:BU65,BT17:BT65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BQ17:BQ65)</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BR13" s="139"/>
-      <c r="BS13" s="139"/>
-      <c r="BT13" s="139"/>
-      <c r="BU13" s="140"/>
+      <c r="BR13" s="141"/>
+      <c r="BS13" s="141"/>
+      <c r="BT13" s="141"/>
+      <c r="BU13" s="142"/>
       <c r="BV13" s="16" t="s">
         <v>15</v>
       </c>
@@ -3173,106 +3173,106 @@
       <c r="K14" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="L14" s="148" t="s">
+      <c r="L14" s="145" t="s">
         <v>17</v>
       </c>
-      <c r="M14" s="149"/>
-      <c r="N14" s="138" cm="1">
+      <c r="M14" s="146"/>
+      <c r="N14" s="140" cm="1">
         <f t="array" ref="N14">SUM(Q17:Q65)+SUM(_xlfn._xlws.FILTER(P17:P65,Q17:Q65=""))+SUM(_xlfn._xlws.FILTER(O17:O65,(P17:P65="")*(Q17:Q65="")))</f>
         <v>674619.25000000012</v>
       </c>
-      <c r="O14" s="139"/>
-      <c r="P14" s="139"/>
-      <c r="Q14" s="139"/>
-      <c r="R14" s="140"/>
-      <c r="S14" s="138" cm="1">
+      <c r="O14" s="141"/>
+      <c r="P14" s="141"/>
+      <c r="Q14" s="141"/>
+      <c r="R14" s="142"/>
+      <c r="S14" s="140" cm="1">
         <f t="array" ref="S14">SUM(V17:V65)+SUM(_xlfn._xlws.FILTER(U17:U65,V17:V65=""))+SUM(_xlfn._xlws.FILTER(T17:T65,(U17:U65="")*(V17:V65="")))</f>
         <v>871752.88</v>
       </c>
-      <c r="T14" s="139"/>
-      <c r="U14" s="139"/>
-      <c r="V14" s="139"/>
-      <c r="W14" s="140"/>
-      <c r="X14" s="138" cm="1">
+      <c r="T14" s="141"/>
+      <c r="U14" s="141"/>
+      <c r="V14" s="141"/>
+      <c r="W14" s="142"/>
+      <c r="X14" s="140" cm="1">
         <f t="array" ref="X14">SUM(AA17:AA65)+SUM(_xlfn._xlws.FILTER(Z17:Z65,AA17:AA65=""))+SUM(_xlfn._xlws.FILTER(Y17:Y65,(Z17:Z65="")*(AA17:AA65="")))</f>
         <v>647579.66999999993</v>
       </c>
-      <c r="Y14" s="139"/>
-      <c r="Z14" s="139"/>
-      <c r="AA14" s="139"/>
-      <c r="AB14" s="140"/>
-      <c r="AC14" s="138" cm="1">
+      <c r="Y14" s="141"/>
+      <c r="Z14" s="141"/>
+      <c r="AA14" s="141"/>
+      <c r="AB14" s="142"/>
+      <c r="AC14" s="140" cm="1">
         <f t="array" ref="AC14">SUM(AF17:AF65)+SUM(_xlfn._xlws.FILTER(AE17:AE65,AF17:AF65=""))+SUM(_xlfn._xlws.FILTER(AD17:AD65,(AE17:AE65="")*(AF17:AF65="")))</f>
         <v>647579.66999999993</v>
       </c>
-      <c r="AD14" s="139"/>
-      <c r="AE14" s="139"/>
-      <c r="AF14" s="139"/>
-      <c r="AG14" s="140"/>
-      <c r="AH14" s="138" cm="1">
+      <c r="AD14" s="141"/>
+      <c r="AE14" s="141"/>
+      <c r="AF14" s="141"/>
+      <c r="AG14" s="142"/>
+      <c r="AH14" s="140" cm="1">
         <f t="array" ref="AH14">SUM(AK17:AK65)+SUM(_xlfn._xlws.FILTER(AJ17:AJ65,AK17:AK65=""))+SUM(_xlfn._xlws.FILTER(AI17:AI65,(AJ17:AJ65="")*(AK17:AK65="")))</f>
         <v>645269.66999999993</v>
       </c>
-      <c r="AI14" s="139"/>
-      <c r="AJ14" s="139"/>
-      <c r="AK14" s="139"/>
-      <c r="AL14" s="140"/>
-      <c r="AM14" s="138" cm="1">
+      <c r="AI14" s="141"/>
+      <c r="AJ14" s="141"/>
+      <c r="AK14" s="141"/>
+      <c r="AL14" s="142"/>
+      <c r="AM14" s="140" cm="1">
         <f t="array" ref="AM14">SUM(AP17:AP65)+SUM(_xlfn._xlws.FILTER(AO17:AO65,AP17:AP65=""))+SUM(_xlfn._xlws.FILTER(AN17:AN65,(AO17:AO65="")*(AP17:AP65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AN14" s="139"/>
-      <c r="AO14" s="139"/>
-      <c r="AP14" s="139"/>
-      <c r="AQ14" s="140"/>
-      <c r="AR14" s="138" cm="1">
+      <c r="AN14" s="141"/>
+      <c r="AO14" s="141"/>
+      <c r="AP14" s="141"/>
+      <c r="AQ14" s="142"/>
+      <c r="AR14" s="140" cm="1">
         <f t="array" ref="AR14">SUM(AU17:AU65)+SUM(_xlfn._xlws.FILTER(AT17:AT65,AU17:AU65=""))+SUM(_xlfn._xlws.FILTER(AS17:AS65,(AT17:AT65="")*(AU17:AU65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AS14" s="139"/>
-      <c r="AT14" s="139"/>
-      <c r="AU14" s="139"/>
-      <c r="AV14" s="140"/>
-      <c r="AW14" s="138" cm="1">
+      <c r="AS14" s="141"/>
+      <c r="AT14" s="141"/>
+      <c r="AU14" s="141"/>
+      <c r="AV14" s="142"/>
+      <c r="AW14" s="140" cm="1">
         <f t="array" ref="AW14">SUM(AZ17:AZ65)+SUM(_xlfn._xlws.FILTER(AY17:AY65,AZ17:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX17:AX65,(AY17:AY65="")*(AZ17:AZ65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="AX14" s="139"/>
-      <c r="AY14" s="139"/>
-      <c r="AZ14" s="139"/>
-      <c r="BA14" s="140"/>
-      <c r="BB14" s="138" cm="1">
+      <c r="AX14" s="141"/>
+      <c r="AY14" s="141"/>
+      <c r="AZ14" s="141"/>
+      <c r="BA14" s="142"/>
+      <c r="BB14" s="140" cm="1">
         <f t="array" ref="BB14">SUM(BE17:BE65)+SUM(_xlfn._xlws.FILTER(BD17:BD65,BE17:BE65=""))+SUM(_xlfn._xlws.FILTER(BC17:BC65,(BD17:BD65="")*(BE17:BE65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BC14" s="139"/>
-      <c r="BD14" s="139"/>
-      <c r="BE14" s="139"/>
-      <c r="BF14" s="140"/>
-      <c r="BG14" s="138" cm="1">
+      <c r="BC14" s="141"/>
+      <c r="BD14" s="141"/>
+      <c r="BE14" s="141"/>
+      <c r="BF14" s="142"/>
+      <c r="BG14" s="140" cm="1">
         <f t="array" ref="BG14">SUM(BJ17:BJ65)+SUM(_xlfn._xlws.FILTER(BI17:BI65,BJ17:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH17:BH65,(BI17:BI65="")*(BJ17:BJ65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BH14" s="139"/>
-      <c r="BI14" s="139"/>
-      <c r="BJ14" s="139"/>
-      <c r="BK14" s="140"/>
-      <c r="BL14" s="138" cm="1">
+      <c r="BH14" s="141"/>
+      <c r="BI14" s="141"/>
+      <c r="BJ14" s="141"/>
+      <c r="BK14" s="142"/>
+      <c r="BL14" s="140" cm="1">
         <f t="array" ref="BL14">SUM(BO17:BO65)+SUM(_xlfn._xlws.FILTER(BN17:BN65,BO17:BO65=""))+SUM(_xlfn._xlws.FILTER(BM17:BM65,(BN17:BN65="")*(BO17:BO65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BM14" s="139"/>
-      <c r="BN14" s="139"/>
-      <c r="BO14" s="139"/>
-      <c r="BP14" s="140"/>
-      <c r="BQ14" s="138" cm="1">
+      <c r="BM14" s="141"/>
+      <c r="BN14" s="141"/>
+      <c r="BO14" s="141"/>
+      <c r="BP14" s="142"/>
+      <c r="BQ14" s="140" cm="1">
         <f t="array" ref="BQ14">SUM(BT17:BT65)+SUM(_xlfn._xlws.FILTER(BS17:BS65,BT17:BT65=""))+SUM(_xlfn._xlws.FILTER(BR17:BR65,(BS17:BS65="")*(BT17:BT65="")))</f>
         <v>635449.66999999993</v>
       </c>
-      <c r="BR14" s="139"/>
-      <c r="BS14" s="139"/>
-      <c r="BT14" s="139"/>
-      <c r="BU14" s="140"/>
+      <c r="BR14" s="141"/>
+      <c r="BS14" s="141"/>
+      <c r="BT14" s="141"/>
+      <c r="BU14" s="142"/>
       <c r="BV14" s="16"/>
       <c r="BW14" s="17"/>
     </row>
@@ -3284,116 +3284,116 @@
         <f>SUBTOTAL(9,K17:K68)</f>
         <v>8537304.5</v>
       </c>
-      <c r="L15" s="150" t="s">
+      <c r="L15" s="147" t="s">
         <v>19</v>
       </c>
-      <c r="M15" s="151"/>
-      <c r="N15" s="141">
+      <c r="M15" s="148"/>
+      <c r="N15" s="149">
         <v>46053</v>
       </c>
-      <c r="O15" s="142" t="s">
+      <c r="O15" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="P15" s="142"/>
-      <c r="Q15" s="142"/>
-      <c r="R15" s="142"/>
-      <c r="S15" s="141" t="s">
+      <c r="P15" s="150"/>
+      <c r="Q15" s="150"/>
+      <c r="R15" s="150"/>
+      <c r="S15" s="149" t="s">
         <v>21</v>
       </c>
-      <c r="T15" s="142"/>
-      <c r="U15" s="142"/>
-      <c r="V15" s="142"/>
-      <c r="W15" s="143"/>
-      <c r="X15" s="141">
+      <c r="T15" s="150"/>
+      <c r="U15" s="150"/>
+      <c r="V15" s="150"/>
+      <c r="W15" s="151"/>
+      <c r="X15" s="149">
         <v>46112</v>
       </c>
-      <c r="Y15" s="142" t="s">
+      <c r="Y15" s="150" t="s">
         <v>22</v>
       </c>
-      <c r="Z15" s="142"/>
-      <c r="AA15" s="142"/>
-      <c r="AB15" s="143"/>
-      <c r="AC15" s="141">
+      <c r="Z15" s="150"/>
+      <c r="AA15" s="150"/>
+      <c r="AB15" s="151"/>
+      <c r="AC15" s="149">
         <v>46142</v>
       </c>
-      <c r="AD15" s="142" t="s">
+      <c r="AD15" s="150" t="s">
         <v>23</v>
       </c>
-      <c r="AE15" s="142"/>
-      <c r="AF15" s="142"/>
-      <c r="AG15" s="143"/>
-      <c r="AH15" s="141">
+      <c r="AE15" s="150"/>
+      <c r="AF15" s="150"/>
+      <c r="AG15" s="151"/>
+      <c r="AH15" s="149">
         <v>46173</v>
       </c>
-      <c r="AI15" s="142" t="s">
+      <c r="AI15" s="150" t="s">
         <v>24</v>
       </c>
-      <c r="AJ15" s="142"/>
-      <c r="AK15" s="142"/>
-      <c r="AL15" s="143"/>
-      <c r="AM15" s="141">
+      <c r="AJ15" s="150"/>
+      <c r="AK15" s="150"/>
+      <c r="AL15" s="151"/>
+      <c r="AM15" s="149">
         <v>46203</v>
       </c>
-      <c r="AN15" s="142" t="s">
+      <c r="AN15" s="150" t="s">
         <v>25</v>
       </c>
-      <c r="AO15" s="142"/>
-      <c r="AP15" s="142"/>
-      <c r="AQ15" s="143"/>
-      <c r="AR15" s="141">
+      <c r="AO15" s="150"/>
+      <c r="AP15" s="150"/>
+      <c r="AQ15" s="151"/>
+      <c r="AR15" s="149">
         <v>46234</v>
       </c>
-      <c r="AS15" s="142" t="s">
+      <c r="AS15" s="150" t="s">
         <v>26</v>
       </c>
-      <c r="AT15" s="142"/>
-      <c r="AU15" s="142"/>
-      <c r="AV15" s="143"/>
-      <c r="AW15" s="141">
+      <c r="AT15" s="150"/>
+      <c r="AU15" s="150"/>
+      <c r="AV15" s="151"/>
+      <c r="AW15" s="149">
         <v>46265</v>
       </c>
-      <c r="AX15" s="142" t="s">
+      <c r="AX15" s="150" t="s">
         <v>27</v>
       </c>
-      <c r="AY15" s="142"/>
-      <c r="AZ15" s="142"/>
-      <c r="BA15" s="143"/>
-      <c r="BB15" s="141">
+      <c r="AY15" s="150"/>
+      <c r="AZ15" s="150"/>
+      <c r="BA15" s="151"/>
+      <c r="BB15" s="149">
         <v>46295</v>
       </c>
-      <c r="BC15" s="142" t="s">
+      <c r="BC15" s="150" t="s">
         <v>28</v>
       </c>
-      <c r="BD15" s="142"/>
-      <c r="BE15" s="142"/>
-      <c r="BF15" s="143"/>
-      <c r="BG15" s="141">
+      <c r="BD15" s="150"/>
+      <c r="BE15" s="150"/>
+      <c r="BF15" s="151"/>
+      <c r="BG15" s="149">
         <v>46326</v>
       </c>
-      <c r="BH15" s="142" t="s">
+      <c r="BH15" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="BI15" s="142"/>
-      <c r="BJ15" s="142"/>
-      <c r="BK15" s="143"/>
-      <c r="BL15" s="141">
+      <c r="BI15" s="150"/>
+      <c r="BJ15" s="150"/>
+      <c r="BK15" s="151"/>
+      <c r="BL15" s="149">
         <v>46356</v>
       </c>
-      <c r="BM15" s="142" t="s">
+      <c r="BM15" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="BN15" s="142"/>
-      <c r="BO15" s="142"/>
-      <c r="BP15" s="143"/>
-      <c r="BQ15" s="141">
+      <c r="BN15" s="150"/>
+      <c r="BO15" s="150"/>
+      <c r="BP15" s="151"/>
+      <c r="BQ15" s="149">
         <v>46387</v>
       </c>
-      <c r="BR15" s="142" t="s">
+      <c r="BR15" s="150" t="s">
         <v>31</v>
       </c>
-      <c r="BS15" s="142"/>
-      <c r="BT15" s="142"/>
-      <c r="BU15" s="143"/>
+      <c r="BS15" s="150"/>
+      <c r="BT15" s="150"/>
+      <c r="BU15" s="151"/>
       <c r="BV15" s="19">
         <f>SUM(BV17:BV65)</f>
         <v>7934948.8299999991</v>
@@ -8798,6 +8798,30 @@
   </sheetData>
   <autoFilter ref="A16:DD71" xr:uid="{177F1DEB-197D-49C6-A2E3-152C1AC7B373}"/>
   <mergeCells count="40">
+    <mergeCell ref="BQ13:BU13"/>
+    <mergeCell ref="BQ15:BU15"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="N13:R13"/>
+    <mergeCell ref="X13:AB13"/>
+    <mergeCell ref="AC13:AG13"/>
+    <mergeCell ref="AH13:AL13"/>
+    <mergeCell ref="AM13:AQ13"/>
+    <mergeCell ref="AR13:AV13"/>
+    <mergeCell ref="AW13:BA13"/>
+    <mergeCell ref="BB13:BF13"/>
+    <mergeCell ref="BG13:BK13"/>
+    <mergeCell ref="BL13:BP13"/>
+    <mergeCell ref="S15:W15"/>
+    <mergeCell ref="N15:R15"/>
+    <mergeCell ref="X15:AB15"/>
+    <mergeCell ref="BB14:BF14"/>
+    <mergeCell ref="BG14:BK14"/>
+    <mergeCell ref="BL14:BP14"/>
+    <mergeCell ref="AC15:AG15"/>
+    <mergeCell ref="AH15:AL15"/>
+    <mergeCell ref="AM15:AQ15"/>
+    <mergeCell ref="AR15:AV15"/>
+    <mergeCell ref="AW15:BA15"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="BQ14:BU14"/>
     <mergeCell ref="L13:M13"/>
@@ -8814,30 +8838,6 @@
     <mergeCell ref="AM14:AQ14"/>
     <mergeCell ref="AR14:AV14"/>
     <mergeCell ref="AW14:BA14"/>
-    <mergeCell ref="BB14:BF14"/>
-    <mergeCell ref="BG14:BK14"/>
-    <mergeCell ref="BL14:BP14"/>
-    <mergeCell ref="AC15:AG15"/>
-    <mergeCell ref="AH15:AL15"/>
-    <mergeCell ref="AM15:AQ15"/>
-    <mergeCell ref="AR15:AV15"/>
-    <mergeCell ref="AW15:BA15"/>
-    <mergeCell ref="BQ13:BU13"/>
-    <mergeCell ref="BQ15:BU15"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="N13:R13"/>
-    <mergeCell ref="X13:AB13"/>
-    <mergeCell ref="AC13:AG13"/>
-    <mergeCell ref="AH13:AL13"/>
-    <mergeCell ref="AM13:AQ13"/>
-    <mergeCell ref="AR13:AV13"/>
-    <mergeCell ref="AW13:BA13"/>
-    <mergeCell ref="BB13:BF13"/>
-    <mergeCell ref="BG13:BK13"/>
-    <mergeCell ref="BL13:BP13"/>
-    <mergeCell ref="S15:W15"/>
-    <mergeCell ref="N15:R15"/>
-    <mergeCell ref="X15:AB15"/>
   </mergeCells>
   <conditionalFormatting sqref="Q17:Q65 V17:V65 AA17:AA65 AF17:AF65 AK17:AK65 AP17:AP65 AU17:AU65 AZ17:AZ65 BE17:BE65 BJ17:BJ65 BO17:BO65 BT17:BT65">
     <cfRule type="expression" dxfId="3" priority="8">
@@ -9029,18 +9029,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9062,14 +9062,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -9083,4 +9075,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add PyYAML to requirements.txt
</commit_message>
<xml_diff>
--- a/data/templates/Ram 2026_Owen Testing.xlsx
+++ b/data/templates/Ram 2026_Owen Testing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/oelkem01_pfizer_com/Documents/SVO/financial-automation-project/data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{7A1710ED-9570-4990-9C3D-DDE87217A9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89BC7557-4DC5-4339-B664-F1819F265931}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{7A1710ED-9570-4990-9C3D-DDE87217A9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFC4670C-9C6F-4343-9F6E-82C4BEE20647}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22920" windowHeight="14250" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="5" r:id="rId1"/>
@@ -2292,12 +2292,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2306,6 +2300,21 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2325,15 +2334,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency 2" xfId="2" xr:uid="{C819F491-96B6-415F-B3EE-ED5A59A1E95E}"/>
@@ -2345,7 +2345,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2359,7 +2359,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFF7C80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2969,10 +2969,10 @@
       <c r="U7" s="14"/>
     </row>
     <row r="8" spans="1:77" x14ac:dyDescent="0.25">
-      <c r="A8" s="138" t="s">
+      <c r="A8" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="139"/>
+      <c r="B8" s="145"/>
       <c r="C8" s="78"/>
       <c r="D8" s="83" t="s">
         <v>8</v>
@@ -3059,112 +3059,112 @@
       <c r="I13" s="68"/>
       <c r="J13" s="68"/>
       <c r="K13" s="72"/>
-      <c r="L13" s="143" t="s">
+      <c r="L13" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="M13" s="144"/>
-      <c r="N13" s="140" cm="1">
+      <c r="M13" s="147"/>
+      <c r="N13" s="138" cm="1">
         <f t="array" ref="N13">SUM(Q17:Q65)+SUM(_xlfn._xlws.FILTER(P17:P65,Q17:Q65=""))+SUM(_xlfn._xlws.FILTER(O17:O65,(P17:P65="")*(Q17:Q65="")))+SUMIFS(R17:R65,Q17:Q65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(N17:N65)</f>
-        <v>410369.37000000011</v>
-      </c>
-      <c r="O13" s="141"/>
-      <c r="P13" s="141"/>
-      <c r="Q13" s="141"/>
-      <c r="R13" s="142"/>
-      <c r="S13" s="140" cm="1">
+        <v>389076.24000000011</v>
+      </c>
+      <c r="O13" s="139"/>
+      <c r="P13" s="139"/>
+      <c r="Q13" s="139"/>
+      <c r="R13" s="140"/>
+      <c r="S13" s="138" cm="1">
         <f t="array" ref="S13">SUM(V17:V65)+SUM(_xlfn._xlws.FILTER(U17:U65,V17:V65=""))+SUM(_xlfn._xlws.FILTER(T17:T65,(U17:U65="")*(V17:V65="")))+SUMIFS(W17:W65,V17:V65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(S17:S65)</f>
         <v>0</v>
       </c>
-      <c r="T13" s="141"/>
-      <c r="U13" s="141"/>
-      <c r="V13" s="141"/>
-      <c r="W13" s="142"/>
-      <c r="X13" s="140" cm="1">
+      <c r="T13" s="139"/>
+      <c r="U13" s="139"/>
+      <c r="V13" s="139"/>
+      <c r="W13" s="140"/>
+      <c r="X13" s="138" cm="1">
         <f t="array" ref="X13">SUM(AA17:AA65)+SUM(_xlfn._xlws.FILTER(Z17:Z65,AA17:AA65=""))+SUM(_xlfn._xlws.FILTER(Y17:Y65,(Z17:Z65="")*(AA17:AA65="")))+SUMIFS(AB17:AB65,AA17:AA65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(X17:X65)</f>
         <v>0</v>
       </c>
-      <c r="Y13" s="141"/>
-      <c r="Z13" s="141"/>
-      <c r="AA13" s="141"/>
-      <c r="AB13" s="142"/>
-      <c r="AC13" s="140" cm="1">
+      <c r="Y13" s="139"/>
+      <c r="Z13" s="139"/>
+      <c r="AA13" s="139"/>
+      <c r="AB13" s="140"/>
+      <c r="AC13" s="138" cm="1">
         <f t="array" ref="AC13">SUM(AF17:AF65)+SUM(_xlfn._xlws.FILTER(AE17:AE65,AF17:AF65=""))+SUM(_xlfn._xlws.FILTER(AD17:AD65,(AE17:AE65="")*(AF17:AF65="")))+SUMIFS(AG17:AG65,AF17:AF65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AC17:AC65)</f>
         <v>0</v>
       </c>
-      <c r="AD13" s="141"/>
-      <c r="AE13" s="141"/>
-      <c r="AF13" s="141"/>
-      <c r="AG13" s="142"/>
-      <c r="AH13" s="140" cm="1">
+      <c r="AD13" s="139"/>
+      <c r="AE13" s="139"/>
+      <c r="AF13" s="139"/>
+      <c r="AG13" s="140"/>
+      <c r="AH13" s="138" cm="1">
         <f t="array" ref="AH13">SUM(AK17:AK65)+SUM(_xlfn._xlws.FILTER(AJ17:AJ65,AK17:AK65=""))+SUM(_xlfn._xlws.FILTER(AI17:AI65,(AJ17:AJ65="")*(AK17:AK65="")))+SUMIFS(AL17:AL65,AK17:AK65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AH17:AH65)</f>
         <v>0</v>
       </c>
-      <c r="AI13" s="141"/>
-      <c r="AJ13" s="141"/>
-      <c r="AK13" s="141"/>
-      <c r="AL13" s="142"/>
-      <c r="AM13" s="140" cm="1">
+      <c r="AI13" s="139"/>
+      <c r="AJ13" s="139"/>
+      <c r="AK13" s="139"/>
+      <c r="AL13" s="140"/>
+      <c r="AM13" s="138" cm="1">
         <f t="array" ref="AM13">SUM(AP17:AP65)+SUM(_xlfn._xlws.FILTER(AO17:AO65,AP17:AP65=""))+SUM(_xlfn._xlws.FILTER(AN17:AN65,(AO17:AO65="")*(AP17:AP65="")))+SUMIFS(AQ17:AQ65,AP17:AP65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AM17:AM65)</f>
         <v>0</v>
       </c>
-      <c r="AN13" s="141"/>
-      <c r="AO13" s="141"/>
-      <c r="AP13" s="141"/>
-      <c r="AQ13" s="142"/>
-      <c r="AR13" s="140" cm="1">
+      <c r="AN13" s="139"/>
+      <c r="AO13" s="139"/>
+      <c r="AP13" s="139"/>
+      <c r="AQ13" s="140"/>
+      <c r="AR13" s="138" cm="1">
         <f t="array" ref="AR13">SUM(AU17:AU65)+SUM(_xlfn._xlws.FILTER(AT17:AT65,AU17:AU65=""))+SUM(_xlfn._xlws.FILTER(AS17:AS65,(AT17:AT65="")*(AU17:AU65="")))+SUMIFS(AV17:AV65,AU17:AU65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AR17:AR65)</f>
         <v>0</v>
       </c>
-      <c r="AS13" s="141"/>
-      <c r="AT13" s="141"/>
-      <c r="AU13" s="141"/>
-      <c r="AV13" s="142"/>
-      <c r="AW13" s="140" cm="1">
+      <c r="AS13" s="139"/>
+      <c r="AT13" s="139"/>
+      <c r="AU13" s="139"/>
+      <c r="AV13" s="140"/>
+      <c r="AW13" s="138" cm="1">
         <f t="array" ref="AW13">SUM(AZ17:AZ65)+SUM(_xlfn._xlws.FILTER(AY17:AY65,AZ17:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX17:AX65,(AY17:AY65="")*(AZ17:AZ65="")))+SUMIFS(BA17:BA65,AZ17:AZ65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(AW17:AW65)</f>
         <v>0</v>
       </c>
-      <c r="AX13" s="141"/>
-      <c r="AY13" s="141"/>
-      <c r="AZ13" s="141"/>
-      <c r="BA13" s="142"/>
-      <c r="BB13" s="140" cm="1">
+      <c r="AX13" s="139"/>
+      <c r="AY13" s="139"/>
+      <c r="AZ13" s="139"/>
+      <c r="BA13" s="140"/>
+      <c r="BB13" s="138" cm="1">
         <f t="array" ref="BB13">SUM(BE17:BE65)+SUM(_xlfn._xlws.FILTER(BD17:BD65,BE17:BE65=""))+SUM(_xlfn._xlws.FILTER(BC17:BC65,(BD17:BD65="")*(BE17:BE65="")))+SUMIFS(BF17:BF65,BE17:BE65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BB17:BB65)</f>
         <v>0</v>
       </c>
-      <c r="BC13" s="141"/>
-      <c r="BD13" s="141"/>
-      <c r="BE13" s="141"/>
-      <c r="BF13" s="142"/>
-      <c r="BG13" s="140" cm="1">
+      <c r="BC13" s="139"/>
+      <c r="BD13" s="139"/>
+      <c r="BE13" s="139"/>
+      <c r="BF13" s="140"/>
+      <c r="BG13" s="138" cm="1">
         <f t="array" ref="BG13">SUM(BJ17:BJ65)+SUM(_xlfn._xlws.FILTER(BI17:BI65,BJ17:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH17:BH65,(BI17:BI65="")*(BJ17:BJ65="")))+SUMIFS(BK17:BK65,BJ17:BJ65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BG17:BG65)</f>
         <v>0</v>
       </c>
-      <c r="BH13" s="141"/>
-      <c r="BI13" s="141"/>
-      <c r="BJ13" s="141"/>
-      <c r="BK13" s="142"/>
-      <c r="BL13" s="140" cm="1">
+      <c r="BH13" s="139"/>
+      <c r="BI13" s="139"/>
+      <c r="BJ13" s="139"/>
+      <c r="BK13" s="140"/>
+      <c r="BL13" s="138" cm="1">
         <f t="array" ref="BL13">SUM(BO17:BO65)+SUM(_xlfn._xlws.FILTER(BN17:BN65,BO17:BO65=""))+SUM(_xlfn._xlws.FILTER(BM17:BM65,(BN17:BN65="")*(BO17:BO65="")))+SUMIFS(BP17:BP65,BO17:BO65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BL17:BL65)</f>
         <v>0</v>
       </c>
-      <c r="BM13" s="141"/>
-      <c r="BN13" s="141"/>
-      <c r="BO13" s="141"/>
-      <c r="BP13" s="142"/>
-      <c r="BQ13" s="140" cm="1">
+      <c r="BM13" s="139"/>
+      <c r="BN13" s="139"/>
+      <c r="BO13" s="139"/>
+      <c r="BP13" s="140"/>
+      <c r="BQ13" s="138" cm="1">
         <f t="array" ref="BQ13">SUM(BT17:BT65)+SUM(_xlfn._xlws.FILTER(BS17:BS65,BT17:BT65=""))+SUM(_xlfn._xlws.FILTER(BR17:BR65,(BS17:BS65="")*(BT17:BT65="")))+SUMIFS(BU17:BU65,BT17:BT65,"&lt;&gt;"&amp;"",$P$17:$P$65,"&lt;&gt;"&amp;"")+SUM(BQ17:BQ65)</f>
         <v>0</v>
       </c>
-      <c r="BR13" s="141"/>
-      <c r="BS13" s="141"/>
-      <c r="BT13" s="141"/>
-      <c r="BU13" s="142"/>
+      <c r="BR13" s="139"/>
+      <c r="BS13" s="139"/>
+      <c r="BT13" s="139"/>
+      <c r="BU13" s="140"/>
       <c r="BV13" s="16" t="s">
         <v>15</v>
       </c>
       <c r="BW13" s="17">
         <f>BW15-BV15</f>
-        <v>-556862.20000000007</v>
+        <v>-535569.07000000007</v>
       </c>
     </row>
     <row r="14" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3180,106 +3180,106 @@
       <c r="K14" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="L14" s="145" t="s">
+      <c r="L14" s="148" t="s">
         <v>17</v>
       </c>
-      <c r="M14" s="146"/>
-      <c r="N14" s="140" cm="1">
+      <c r="M14" s="149"/>
+      <c r="N14" s="138" cm="1">
         <f t="array" ref="N14">SUM(Q17:Q65)+SUM(_xlfn._xlws.FILTER(P17:P65,Q17:Q65=""))+SUM(_xlfn._xlws.FILTER(O17:O65,(P17:P65="")*(Q17:Q65="")))</f>
-        <v>556862.20000000007</v>
-      </c>
-      <c r="O14" s="141"/>
-      <c r="P14" s="141"/>
-      <c r="Q14" s="141"/>
-      <c r="R14" s="142"/>
-      <c r="S14" s="140" cm="1">
+        <v>535569.07000000007</v>
+      </c>
+      <c r="O14" s="139"/>
+      <c r="P14" s="139"/>
+      <c r="Q14" s="139"/>
+      <c r="R14" s="140"/>
+      <c r="S14" s="138" cm="1">
         <f t="array" ref="S14">SUM(V17:V65)+SUM(_xlfn._xlws.FILTER(U17:U65,V17:V65=""))+SUM(_xlfn._xlws.FILTER(T17:T65,(U17:U65="")*(V17:V65="")))</f>
         <v>0</v>
       </c>
-      <c r="T14" s="141"/>
-      <c r="U14" s="141"/>
-      <c r="V14" s="141"/>
-      <c r="W14" s="142"/>
-      <c r="X14" s="140" cm="1">
+      <c r="T14" s="139"/>
+      <c r="U14" s="139"/>
+      <c r="V14" s="139"/>
+      <c r="W14" s="140"/>
+      <c r="X14" s="138" cm="1">
         <f t="array" ref="X14">SUM(AA17:AA65)+SUM(_xlfn._xlws.FILTER(Z17:Z65,AA17:AA65=""))+SUM(_xlfn._xlws.FILTER(Y17:Y65,(Z17:Z65="")*(AA17:AA65="")))</f>
         <v>0</v>
       </c>
-      <c r="Y14" s="141"/>
-      <c r="Z14" s="141"/>
-      <c r="AA14" s="141"/>
-      <c r="AB14" s="142"/>
-      <c r="AC14" s="140" cm="1">
+      <c r="Y14" s="139"/>
+      <c r="Z14" s="139"/>
+      <c r="AA14" s="139"/>
+      <c r="AB14" s="140"/>
+      <c r="AC14" s="138" cm="1">
         <f t="array" ref="AC14">SUM(AF17:AF65)+SUM(_xlfn._xlws.FILTER(AE17:AE65,AF17:AF65=""))+SUM(_xlfn._xlws.FILTER(AD17:AD65,(AE17:AE65="")*(AF17:AF65="")))</f>
         <v>0</v>
       </c>
-      <c r="AD14" s="141"/>
-      <c r="AE14" s="141"/>
-      <c r="AF14" s="141"/>
-      <c r="AG14" s="142"/>
-      <c r="AH14" s="140" cm="1">
+      <c r="AD14" s="139"/>
+      <c r="AE14" s="139"/>
+      <c r="AF14" s="139"/>
+      <c r="AG14" s="140"/>
+      <c r="AH14" s="138" cm="1">
         <f t="array" ref="AH14">SUM(AK17:AK65)+SUM(_xlfn._xlws.FILTER(AJ17:AJ65,AK17:AK65=""))+SUM(_xlfn._xlws.FILTER(AI17:AI65,(AJ17:AJ65="")*(AK17:AK65="")))</f>
         <v>0</v>
       </c>
-      <c r="AI14" s="141"/>
-      <c r="AJ14" s="141"/>
-      <c r="AK14" s="141"/>
-      <c r="AL14" s="142"/>
-      <c r="AM14" s="140" cm="1">
+      <c r="AI14" s="139"/>
+      <c r="AJ14" s="139"/>
+      <c r="AK14" s="139"/>
+      <c r="AL14" s="140"/>
+      <c r="AM14" s="138" cm="1">
         <f t="array" ref="AM14">SUM(AP17:AP65)+SUM(_xlfn._xlws.FILTER(AO17:AO65,AP17:AP65=""))+SUM(_xlfn._xlws.FILTER(AN17:AN65,(AO17:AO65="")*(AP17:AP65="")))</f>
         <v>0</v>
       </c>
-      <c r="AN14" s="141"/>
-      <c r="AO14" s="141"/>
-      <c r="AP14" s="141"/>
-      <c r="AQ14" s="142"/>
-      <c r="AR14" s="140" cm="1">
+      <c r="AN14" s="139"/>
+      <c r="AO14" s="139"/>
+      <c r="AP14" s="139"/>
+      <c r="AQ14" s="140"/>
+      <c r="AR14" s="138" cm="1">
         <f t="array" ref="AR14">SUM(AU17:AU65)+SUM(_xlfn._xlws.FILTER(AT17:AT65,AU17:AU65=""))+SUM(_xlfn._xlws.FILTER(AS17:AS65,(AT17:AT65="")*(AU17:AU65="")))</f>
         <v>0</v>
       </c>
-      <c r="AS14" s="141"/>
-      <c r="AT14" s="141"/>
-      <c r="AU14" s="141"/>
-      <c r="AV14" s="142"/>
-      <c r="AW14" s="140" cm="1">
+      <c r="AS14" s="139"/>
+      <c r="AT14" s="139"/>
+      <c r="AU14" s="139"/>
+      <c r="AV14" s="140"/>
+      <c r="AW14" s="138" cm="1">
         <f t="array" ref="AW14">SUM(AZ17:AZ65)+SUM(_xlfn._xlws.FILTER(AY17:AY65,AZ17:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX17:AX65,(AY17:AY65="")*(AZ17:AZ65="")))</f>
         <v>0</v>
       </c>
-      <c r="AX14" s="141"/>
-      <c r="AY14" s="141"/>
-      <c r="AZ14" s="141"/>
-      <c r="BA14" s="142"/>
-      <c r="BB14" s="140" cm="1">
+      <c r="AX14" s="139"/>
+      <c r="AY14" s="139"/>
+      <c r="AZ14" s="139"/>
+      <c r="BA14" s="140"/>
+      <c r="BB14" s="138" cm="1">
         <f t="array" ref="BB14">SUM(BE17:BE65)+SUM(_xlfn._xlws.FILTER(BD17:BD65,BE17:BE65=""))+SUM(_xlfn._xlws.FILTER(BC17:BC65,(BD17:BD65="")*(BE17:BE65="")))</f>
         <v>0</v>
       </c>
-      <c r="BC14" s="141"/>
-      <c r="BD14" s="141"/>
-      <c r="BE14" s="141"/>
-      <c r="BF14" s="142"/>
-      <c r="BG14" s="140" cm="1">
+      <c r="BC14" s="139"/>
+      <c r="BD14" s="139"/>
+      <c r="BE14" s="139"/>
+      <c r="BF14" s="140"/>
+      <c r="BG14" s="138" cm="1">
         <f t="array" ref="BG14">SUM(BJ17:BJ65)+SUM(_xlfn._xlws.FILTER(BI17:BI65,BJ17:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH17:BH65,(BI17:BI65="")*(BJ17:BJ65="")))</f>
         <v>0</v>
       </c>
-      <c r="BH14" s="141"/>
-      <c r="BI14" s="141"/>
-      <c r="BJ14" s="141"/>
-      <c r="BK14" s="142"/>
-      <c r="BL14" s="140" cm="1">
+      <c r="BH14" s="139"/>
+      <c r="BI14" s="139"/>
+      <c r="BJ14" s="139"/>
+      <c r="BK14" s="140"/>
+      <c r="BL14" s="138" cm="1">
         <f t="array" ref="BL14">SUM(BO17:BO65)+SUM(_xlfn._xlws.FILTER(BN17:BN65,BO17:BO65=""))+SUM(_xlfn._xlws.FILTER(BM17:BM65,(BN17:BN65="")*(BO17:BO65="")))</f>
         <v>0</v>
       </c>
-      <c r="BM14" s="141"/>
-      <c r="BN14" s="141"/>
-      <c r="BO14" s="141"/>
-      <c r="BP14" s="142"/>
-      <c r="BQ14" s="140" cm="1">
+      <c r="BM14" s="139"/>
+      <c r="BN14" s="139"/>
+      <c r="BO14" s="139"/>
+      <c r="BP14" s="140"/>
+      <c r="BQ14" s="138" cm="1">
         <f t="array" ref="BQ14">SUM(BT17:BT65)+SUM(_xlfn._xlws.FILTER(BS17:BS65,BT17:BT65=""))+SUM(_xlfn._xlws.FILTER(BR17:BR65,(BS17:BS65="")*(BT17:BT65="")))</f>
         <v>0</v>
       </c>
-      <c r="BR14" s="141"/>
-      <c r="BS14" s="141"/>
-      <c r="BT14" s="141"/>
-      <c r="BU14" s="142"/>
+      <c r="BR14" s="139"/>
+      <c r="BS14" s="139"/>
+      <c r="BT14" s="139"/>
+      <c r="BU14" s="140"/>
       <c r="BV14" s="16"/>
       <c r="BW14" s="17"/>
     </row>
@@ -3291,119 +3291,119 @@
         <f>SUBTOTAL(9,K17:K68)</f>
         <v>8537304.5</v>
       </c>
-      <c r="L15" s="147" t="s">
+      <c r="L15" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="M15" s="148"/>
-      <c r="N15" s="149">
+      <c r="M15" s="151"/>
+      <c r="N15" s="141">
         <v>46053</v>
       </c>
-      <c r="O15" s="150" t="s">
+      <c r="O15" s="142" t="s">
         <v>20</v>
       </c>
-      <c r="P15" s="150"/>
-      <c r="Q15" s="150"/>
-      <c r="R15" s="150"/>
-      <c r="S15" s="149" t="s">
+      <c r="P15" s="142"/>
+      <c r="Q15" s="142"/>
+      <c r="R15" s="142"/>
+      <c r="S15" s="141" t="s">
         <v>21</v>
       </c>
-      <c r="T15" s="150"/>
-      <c r="U15" s="150"/>
-      <c r="V15" s="150"/>
-      <c r="W15" s="151"/>
-      <c r="X15" s="149">
+      <c r="T15" s="142"/>
+      <c r="U15" s="142"/>
+      <c r="V15" s="142"/>
+      <c r="W15" s="143"/>
+      <c r="X15" s="141">
         <v>46112</v>
       </c>
-      <c r="Y15" s="150" t="s">
+      <c r="Y15" s="142" t="s">
         <v>22</v>
       </c>
-      <c r="Z15" s="150"/>
-      <c r="AA15" s="150"/>
-      <c r="AB15" s="151"/>
-      <c r="AC15" s="149">
+      <c r="Z15" s="142"/>
+      <c r="AA15" s="142"/>
+      <c r="AB15" s="143"/>
+      <c r="AC15" s="141">
         <v>46142</v>
       </c>
-      <c r="AD15" s="150" t="s">
+      <c r="AD15" s="142" t="s">
         <v>23</v>
       </c>
-      <c r="AE15" s="150"/>
-      <c r="AF15" s="150"/>
-      <c r="AG15" s="151"/>
-      <c r="AH15" s="149">
+      <c r="AE15" s="142"/>
+      <c r="AF15" s="142"/>
+      <c r="AG15" s="143"/>
+      <c r="AH15" s="141">
         <v>46173</v>
       </c>
-      <c r="AI15" s="150" t="s">
+      <c r="AI15" s="142" t="s">
         <v>24</v>
       </c>
-      <c r="AJ15" s="150"/>
-      <c r="AK15" s="150"/>
-      <c r="AL15" s="151"/>
-      <c r="AM15" s="149">
+      <c r="AJ15" s="142"/>
+      <c r="AK15" s="142"/>
+      <c r="AL15" s="143"/>
+      <c r="AM15" s="141">
         <v>46203</v>
       </c>
-      <c r="AN15" s="150" t="s">
+      <c r="AN15" s="142" t="s">
         <v>25</v>
       </c>
-      <c r="AO15" s="150"/>
-      <c r="AP15" s="150"/>
-      <c r="AQ15" s="151"/>
-      <c r="AR15" s="149">
+      <c r="AO15" s="142"/>
+      <c r="AP15" s="142"/>
+      <c r="AQ15" s="143"/>
+      <c r="AR15" s="141">
         <v>46234</v>
       </c>
-      <c r="AS15" s="150" t="s">
+      <c r="AS15" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="AT15" s="150"/>
-      <c r="AU15" s="150"/>
-      <c r="AV15" s="151"/>
-      <c r="AW15" s="149">
+      <c r="AT15" s="142"/>
+      <c r="AU15" s="142"/>
+      <c r="AV15" s="143"/>
+      <c r="AW15" s="141">
         <v>46265</v>
       </c>
-      <c r="AX15" s="150" t="s">
+      <c r="AX15" s="142" t="s">
         <v>27</v>
       </c>
-      <c r="AY15" s="150"/>
-      <c r="AZ15" s="150"/>
-      <c r="BA15" s="151"/>
-      <c r="BB15" s="149">
+      <c r="AY15" s="142"/>
+      <c r="AZ15" s="142"/>
+      <c r="BA15" s="143"/>
+      <c r="BB15" s="141">
         <v>46295</v>
       </c>
-      <c r="BC15" s="150" t="s">
+      <c r="BC15" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="BD15" s="150"/>
-      <c r="BE15" s="150"/>
-      <c r="BF15" s="151"/>
-      <c r="BG15" s="149">
+      <c r="BD15" s="142"/>
+      <c r="BE15" s="142"/>
+      <c r="BF15" s="143"/>
+      <c r="BG15" s="141">
         <v>46326</v>
       </c>
-      <c r="BH15" s="150" t="s">
+      <c r="BH15" s="142" t="s">
         <v>29</v>
       </c>
-      <c r="BI15" s="150"/>
-      <c r="BJ15" s="150"/>
-      <c r="BK15" s="151"/>
-      <c r="BL15" s="149">
+      <c r="BI15" s="142"/>
+      <c r="BJ15" s="142"/>
+      <c r="BK15" s="143"/>
+      <c r="BL15" s="141">
         <v>46356</v>
       </c>
-      <c r="BM15" s="150" t="s">
+      <c r="BM15" s="142" t="s">
         <v>30</v>
       </c>
-      <c r="BN15" s="150"/>
-      <c r="BO15" s="150"/>
-      <c r="BP15" s="151"/>
-      <c r="BQ15" s="149">
+      <c r="BN15" s="142"/>
+      <c r="BO15" s="142"/>
+      <c r="BP15" s="143"/>
+      <c r="BQ15" s="141">
         <v>46387</v>
       </c>
-      <c r="BR15" s="150" t="s">
+      <c r="BR15" s="142" t="s">
         <v>31</v>
       </c>
-      <c r="BS15" s="150"/>
-      <c r="BT15" s="150"/>
-      <c r="BU15" s="151"/>
+      <c r="BS15" s="142"/>
+      <c r="BT15" s="142"/>
+      <c r="BU15" s="143"/>
       <c r="BV15" s="19">
         <f>SUM(BV17:BV65)</f>
-        <v>556862.20000000007</v>
+        <v>535569.07000000007</v>
       </c>
       <c r="BW15" s="20"/>
       <c r="BY15" s="15"/>
@@ -3681,15 +3681,9 @@
       <c r="N17" s="91">
         <v>0</v>
       </c>
-      <c r="O17" s="34">
-        <v>10975</v>
-      </c>
-      <c r="P17" s="34">
-        <v>11347.01</v>
-      </c>
-      <c r="Q17" s="82">
-        <v>10656.33</v>
-      </c>
+      <c r="O17" s="34"/>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="82"/>
       <c r="R17" s="36"/>
       <c r="S17" s="35"/>
       <c r="T17" s="34"/>
@@ -3748,7 +3742,7 @@
       <c r="BU17" s="42"/>
       <c r="BV17" s="35">
         <f t="shared" ref="BV17:BV65" si="0">SUM(IF(Q17&lt;&gt;"",Q17,IF(P17&lt;&gt;"",P17,O17)),IF(V17&lt;&gt;"",V17,IF(U17&lt;&gt;"",U17,T17)),IF(AA17&lt;&gt;"",AA17,IF(Z17&lt;&gt;"",Z17,Y17)),IF(AF17&lt;&gt;"",AF17,IF(AE17&lt;&gt;"",AE17,AD17)),IF(AK17&lt;&gt;"",AK17,IF(AJ17&lt;&gt;"",AJ17,AI17)),IF(AP17&lt;&gt;"",AP17,IF(AO17&lt;&gt;"",AO17,AN17)),IF(AU17&lt;&gt;"",AU17,IF(AT17&lt;&gt;"",AT17,AS17)),IF(AZ17&lt;&gt;"",AZ17,IF(AY17&lt;&gt;"",AY17,AX17)),IF(BE17&lt;&gt;"",BE17,IF(BD17&lt;&gt;"",BD17,BC17)),IF(BJ17&lt;&gt;"",BJ17,IF(BI17&lt;&gt;"",BI17,BH17)),IF(BO17&lt;&gt;"",BO17,IF(BN17&lt;&gt;"",BN17,BM17)),IF(BT17&lt;&gt;"",BT17,IF(BS17&lt;&gt;"",BS17,BR17)))</f>
-        <v>10656.33</v>
+        <v>0</v>
       </c>
       <c r="BW17" s="49"/>
       <c r="BX17" s="50"/>
@@ -3796,15 +3790,9 @@
       <c r="N18" s="92">
         <v>0</v>
       </c>
-      <c r="O18" s="39">
-        <v>10296</v>
-      </c>
-      <c r="P18" s="39">
-        <v>10548.89</v>
-      </c>
-      <c r="Q18" s="85">
-        <v>10636.8</v>
-      </c>
+      <c r="O18" s="39"/>
+      <c r="P18" s="39"/>
+      <c r="Q18" s="85"/>
       <c r="R18" s="41"/>
       <c r="S18" s="40"/>
       <c r="T18" s="39"/>
@@ -3863,7 +3851,7 @@
       <c r="BU18" s="42"/>
       <c r="BV18" s="35">
         <f t="shared" si="0"/>
-        <v>10636.8</v>
+        <v>0</v>
       </c>
       <c r="BW18" s="51"/>
       <c r="BX18" s="52"/>
@@ -8334,6 +8322,30 @@
   </sheetData>
   <autoFilter ref="A16:DD71" xr:uid="{177F1DEB-197D-49C6-A2E3-152C1AC7B373}"/>
   <mergeCells count="40">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="BQ14:BU14"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="BB15:BF15"/>
+    <mergeCell ref="BG15:BK15"/>
+    <mergeCell ref="BL15:BP15"/>
+    <mergeCell ref="N14:R14"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="X14:AB14"/>
+    <mergeCell ref="AC14:AG14"/>
+    <mergeCell ref="AH14:AL14"/>
+    <mergeCell ref="AM14:AQ14"/>
+    <mergeCell ref="AR14:AV14"/>
+    <mergeCell ref="AW14:BA14"/>
+    <mergeCell ref="BB14:BF14"/>
+    <mergeCell ref="BG14:BK14"/>
+    <mergeCell ref="BL14:BP14"/>
+    <mergeCell ref="AC15:AG15"/>
+    <mergeCell ref="AH15:AL15"/>
+    <mergeCell ref="AM15:AQ15"/>
+    <mergeCell ref="AR15:AV15"/>
+    <mergeCell ref="AW15:BA15"/>
     <mergeCell ref="BQ13:BU13"/>
     <mergeCell ref="BQ15:BU15"/>
     <mergeCell ref="S13:W13"/>
@@ -8350,54 +8362,30 @@
     <mergeCell ref="S15:W15"/>
     <mergeCell ref="N15:R15"/>
     <mergeCell ref="X15:AB15"/>
-    <mergeCell ref="BB14:BF14"/>
-    <mergeCell ref="BG14:BK14"/>
-    <mergeCell ref="BL14:BP14"/>
-    <mergeCell ref="AC15:AG15"/>
-    <mergeCell ref="AH15:AL15"/>
-    <mergeCell ref="AM15:AQ15"/>
-    <mergeCell ref="AR15:AV15"/>
-    <mergeCell ref="AW15:BA15"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="BQ14:BU14"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="BB15:BF15"/>
-    <mergeCell ref="BG15:BK15"/>
-    <mergeCell ref="BL15:BP15"/>
-    <mergeCell ref="N14:R14"/>
-    <mergeCell ref="S14:W14"/>
-    <mergeCell ref="X14:AB14"/>
-    <mergeCell ref="AC14:AG14"/>
-    <mergeCell ref="AH14:AL14"/>
-    <mergeCell ref="AM14:AQ14"/>
-    <mergeCell ref="AR14:AV14"/>
-    <mergeCell ref="AW14:BA14"/>
   </mergeCells>
-  <conditionalFormatting sqref="Q65 V17:V65 AA17:AA65 AF17:AF65 AK17:AK65 AP17:AP65 AU17:AU65 AZ17:AZ65 BE17:BE65 BJ17:BJ65 BO17:BO65 BT17:BT65">
-    <cfRule type="expression" dxfId="4" priority="9">
+  <conditionalFormatting sqref="Q17:Q65">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>IF(AND(P17&gt;0,Q17=0),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="V17:V65 AA17:AA65 AF17:AF65 AK17:AK65 AP17:AP65 AU17:AU65 AZ17:AZ65 BE17:BE65 BJ17:BJ65 BO17:BO65 BT17:BT65">
+    <cfRule type="expression" dxfId="3" priority="9">
+      <formula>IF(AND(U17&gt;0,V17=0),TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="BT12 V17:X65 AB17:AC65 AG17:AH65 AL17:AM65 AQ17:AR65 AV17:AW65 BA17:BB65 BF17:BG65 BK17:BL65 BP17:BQ65 BU17:BU65">
-    <cfRule type="expression" dxfId="3" priority="10">
+    <cfRule type="expression" dxfId="2" priority="10">
       <formula>IF(AND(U12&lt;&gt;"",V12="",TODAY()&gt;DATE(YEAR(TODAY()),MONTH(DATEVALUE("1-"&amp;LEFT(#REF!,3)&amp;"-1900")),20)),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BV17:BV64">
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="greaterThan">
       <formula>90%*$K$17</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BW13:BW14">
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>IF(BW13&lt;0,TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q17:Q64">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>IF(AND(P17&gt;0,Q17=0),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8408,6 +8396,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100705CE5A564F40946AECC6EBE58791375" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8ba3a2bde39cc3ca0702cdfcb4eca37d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca7236cb-6f9c-48f7-87fd-cb400629eee9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="22de7e6ac394ce7397beb0dba85b4d79" ns2:_="">
     <xsd:import namespace="ca7236cb-6f9c-48f7-87fd-cb400629eee9"/>
@@ -8569,35 +8572,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD946F0F-13D5-444C-A93C-86A02D792EE0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca7236cb-6f9c-48f7-87fd-cb400629eee9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8619,9 +8597,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD946F0F-13D5-444C-A93C-86A02D792EE0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca7236cb-6f9c-48f7-87fd-cb400629eee9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>